<commit_message>
EU list: add large European manufacturers sheet (Italy, Germany, UK, Spain, Sweden)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013pAYVPcDWTLeuLdwVsKmmQ
</commit_message>
<xml_diff>
--- a/suppliers_us/Aldera_EU_manufacturers_2026-10-29.xlsx
+++ b/suppliers_us/Aldera_EU_manufacturers_2026-10-29.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Заводы ЕС" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Важно" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Крупные заводы Европы" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Важно" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -954,6 +955,552 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Страна</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Компания</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Город</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Что делают</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Размер / минимум</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Реестр NSF/ANSI 455-2</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Вывод</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Италия</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Ourvita (Farmaceutici Procemsa)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Nichelino (Турин)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Капсулы, таблетки, саше, стики; только для третьих лиц</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Позиционирует себя как крупнейший CDMO добавок в Европе</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Есть (производство, инкапсуляция)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Первый кандидат на масштаб</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Италия</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Biofarma Group</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Mereto di Tomba (Удине)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Твёрдые формы, саше, стики, порошки; только для третьих лиц</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Крупный, глобальный</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Есть (производство)</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Первый кандидат на масштаб</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Италия</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Labomar</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Istrana (Тревизо)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Капсулы, таблетки, саше; публичная компания</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Крупный</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Нет в выгрузке</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Запросить; данных в поиске нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Италия</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Erbozeta</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Сан-Марино</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Таблетки, капсулы, саше, стики</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Средний-крупный</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Нет в выгрузке</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Запасной</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Германия</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Alphacaps</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Thoßfell (Саксония)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Капсулы, своя марка под ключ</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>200-499 сотрудников; GMP, IFS</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Нет в выгрузке</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Главный немецкий кандидат по капсулам</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Германия</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Wellma Europe (бывш. Private Label Factory)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Recklinghausen, Hamburg</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Капсулы HPMC и желатин, таблетки, порошки, софтгели, гамми</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>15 заводов в 9 странах</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Нет в выгрузке</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Крупная группа; есть завод и в Нидерландах (Duiven)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Германия</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Goerlich Pharma</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Edling (Бавария)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Капсулы, саше</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Минимум 500 000 капсул или саше</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Нет в выгрузке</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Только на масштаб</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Великобритания</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Cultech</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Port Talbot (Уэльс)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Капсулы, порошки, пробиотики</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Несколько площадок</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Есть (производство, инкапсуляция)</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Не ЕС; пошлина США на UK ниже. Надпись Made in UK</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Великобритания</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Supplement Factory</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Ashford (Кент)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Капсулы, порошки, своя марка</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Средний</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Есть (производство)</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Работает с малыми брендами</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Испания</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>MARNYS (Martínez Nieto)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Картахена</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Капсулы, софтгели</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>GMP, IFS; заявляют регистрацию FDA; 60-70 стран</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Нет в выгрузке</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Из нашего прошлого разбора: лучший испанский для США</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Испания</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Industrial Farmacéutica Cantabria</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Torrejón de Ardoz (Мадрид)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Капсулы, порошки</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Фармацевтический</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Есть (производство, инкапсуляция)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Проверить, работают ли с добавками под чужой маркой</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Швеция</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Legosan</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Kumla</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Капсулы, гамми, порошки</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Средний</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Есть (производство, инкапсуляция)</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Запасной</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>